<commit_message>
Little reorganization and added project related files and docs for Spring 2022 - Pratik
</commit_message>
<xml_diff>
--- a/spring-2022/Attendance.xlsx
+++ b/spring-2022/Attendance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24729"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VIP\Github_repos\vip-nlp\spring-2022\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D18FC74F-0B23-4AEF-907A-0BC647D7E238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27D130E-D55A-44AA-834D-5213D3CA35F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -504,7 +504,7 @@
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
+      <c r="D5" s="6"/>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
@@ -534,7 +534,7 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
+      <c r="D6" s="6"/>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>

</xml_diff>

<commit_message>
Adding subteam presentation 2
</commit_message>
<xml_diff>
--- a/spring-2022/Attendance.xlsx
+++ b/spring-2022/Attendance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VIP\Github_repos\vip-nlp\spring-2022\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27D130E-D55A-44AA-834D-5213D3CA35F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E747B5-25DE-4B2A-AACB-3CF5B32A0440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -417,7 +417,7 @@
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
+      <c r="G2" s="6"/>
       <c r="H2" s="8"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
@@ -537,7 +537,7 @@
       <c r="D6" s="6"/>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
+      <c r="G6" s="6"/>
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
@@ -568,7 +568,7 @@
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
+      <c r="H7" s="6"/>
       <c r="I7" s="8"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
@@ -628,7 +628,7 @@
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
+      <c r="H9" s="6"/>
       <c r="I9" s="8"/>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>

</xml_diff>

<commit_message>
Final Presentation + Attendance
</commit_message>
<xml_diff>
--- a/spring-2022/Attendance.xlsx
+++ b/spring-2022/Attendance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VIP\Github_repos\vip-nlp\spring-2022\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E747B5-25DE-4B2A-AACB-3CF5B32A0440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD35BFD5-617B-4DAD-8260-0996B6125A5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -390,12 +390,8 @@
       <c r="M1" s="2">
         <v>44665</v>
       </c>
-      <c r="N1" s="2">
-        <v>44672</v>
-      </c>
-      <c r="O1" s="2">
-        <v>44679</v>
-      </c>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
       <c r="P1" s="3"/>
       <c r="Q1" s="3"/>
       <c r="R1" s="3"/>
@@ -422,7 +418,7 @@
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
+      <c r="L2" s="6"/>
       <c r="M2" s="7"/>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
@@ -449,7 +445,7 @@
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
-      <c r="I3" s="8"/>
+      <c r="I3" s="6"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
@@ -481,7 +477,7 @@
       <c r="H4" s="7"/>
       <c r="I4" s="8"/>
       <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
+      <c r="K4" s="6"/>
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
@@ -513,7 +509,7 @@
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
-      <c r="M5" s="7"/>
+      <c r="M5" s="6"/>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
       <c r="P5" s="3"/>
@@ -542,7 +538,7 @@
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
+      <c r="L6" s="6"/>
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
@@ -571,9 +567,9 @@
       <c r="H7" s="6"/>
       <c r="I7" s="8"/>
       <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
+      <c r="K7" s="6"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
+      <c r="M7" s="6"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
       <c r="P7" s="3"/>

</xml_diff>